<commit_message>
Created basics for hex based system
</commit_message>
<xml_diff>
--- a/worklog.xlsx
+++ b/worklog.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Seth\Desktop\Programming\Unity\RPGTemplate\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502074DC-0713-44B4-8BC4-D44F949E267F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,31 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Total Hours</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>1:55 - 3:25</t>
+  </si>
+  <si>
+    <t>Created repository and initial setup</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -37,7 +66,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +74,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +370,45 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="36.109375" customWidth="1"/>
+    <col min="2" max="2" width="25.77734375" customWidth="1"/>
+    <col min="3" max="3" width="20.77734375" customWidth="1"/>
+    <col min="4" max="4" width="31.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>46058</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>1.5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Created basics for Hex Math, Line drawing, and basic hex calculations
</commit_message>
<xml_diff>
--- a/worklog.xlsx
+++ b/worklog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Seth\Desktop\Programming\Unity\RPGTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45E7B88-E627-42C1-95D9-DB4871A080D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5E770A-BAEB-4C92-8A39-67CE3B7D5A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Date</t>
   </si>
@@ -46,6 +46,15 @@
   </si>
   <si>
     <t>6:00-7:00</t>
+  </si>
+  <si>
+    <t>Began creation of Hexagon system. Had to restart due to several errors.</t>
+  </si>
+  <si>
+    <t>7:10-8:10</t>
+  </si>
+  <si>
+    <t>Created basics for Hex Math, Line drawing, and basic hex calculations</t>
   </si>
 </sst>
 </file>
@@ -375,16 +384,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36.109375" customWidth="1"/>
-    <col min="2" max="2" width="25.77734375" customWidth="1"/>
-    <col min="3" max="3" width="20.77734375" customWidth="1"/>
-    <col min="4" max="4" width="31.109375" customWidth="1"/>
+    <col min="1" max="1" width="36.08984375" customWidth="1"/>
+    <col min="2" max="2" width="25.81640625" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" customWidth="1"/>
+    <col min="4" max="4" width="31.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -398,7 +407,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>46058</v>
       </c>
@@ -412,7 +421,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>46074</v>
       </c>
@@ -421,6 +430,23 @@
       </c>
       <c r="C3">
         <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="1">
+        <v>46079</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made changes to hexTile, HexGrid, and Hex to reflect a custom editor
</commit_message>
<xml_diff>
--- a/worklog.xlsx
+++ b/worklog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Seth\Desktop\Programming\Unity\RPGTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5E770A-BAEB-4C92-8A39-67CE3B7D5A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0635B1B-0FE5-4107-9BC3-F264659D8B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25840" windowHeight="15520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Date</t>
   </si>
@@ -55,6 +55,12 @@
   </si>
   <si>
     <t>Created basics for Hex Math, Line drawing, and basic hex calculations</t>
+  </si>
+  <si>
+    <t>11:00-12:45</t>
+  </si>
+  <si>
+    <t>Made more tilemap things. Worked on creating Unity Tilemap</t>
   </si>
 </sst>
 </file>
@@ -384,7 +390,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36.08984375" customWidth="1"/>
@@ -449,6 +455,20 @@
         <v>9</v>
       </c>
     </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="1">
+        <v>46080</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <v>1.75</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Pre-breaking my project for Claude's delight
</commit_message>
<xml_diff>
--- a/worklog.xlsx
+++ b/worklog.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Seth\Desktop\Programming\Unity\RPGTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10EE934F-309D-4CE0-A164-4A6DD79217F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E3CF3B-ED01-4BDF-9F33-60F36A172AD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25840" windowHeight="15520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Date</t>
   </si>
@@ -33,9 +44,6 @@
     <t>Time</t>
   </si>
   <si>
-    <t>Total Hours</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -73,6 +81,12 @@
   </si>
   <si>
     <t>Made the AI as well as player interaction.</t>
+  </si>
+  <si>
+    <t>6:45-7:45</t>
+  </si>
+  <si>
+    <t>Spent the full time fixing a problem with tile spacing</t>
   </si>
 </sst>
 </file>
@@ -403,7 +417,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36.08984375" customWidth="1"/>
@@ -419,11 +433,12 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="2">
+        <f>SUM(C2:C100)</f>
+        <v>9.5</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -431,13 +446,13 @@
         <v>46058</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2">
         <v>1.5</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -445,13 +460,13 @@
         <v>46074</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -459,13 +474,13 @@
         <v>46079</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -473,13 +488,13 @@
         <v>46080</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>1.75</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -487,13 +502,13 @@
         <v>46090</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6">
         <v>1.5</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -501,13 +516,27 @@
         <v>46091</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C7">
         <v>1.75</v>
       </c>
       <c r="D7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B8" t="s">
         <v>15</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>